<commit_message>
ajout léa modif tableur excel
</commit_message>
<xml_diff>
--- a/data/climate_data/SuppData.xlsx
+++ b/data/climate_data/SuppData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN.RDS-PRET-0218\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN.RDS-PRET-0218\Desktop\Agrocampus Ouest\M2\Projet ingénieur\meteo_vs_rendement\data\climate_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98316C89-43A7-4429-830E-8C62C60AFA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0BBA77-FF74-4513-814B-48307828504B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{13E9D6FB-1915-45C5-BF12-168D097CE999}"/>
   </bookViews>
@@ -1483,19 +1483,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -14894,5 +14894,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>